<commit_message>
corpus: publish trustworthy audited bundles
Add atomic publication metadata, strict artifact auditing, resumable zero-API migration, honest quality metrics, and republish the 2025-2026 converted corpus as verified modern bundles.
</commit_message>
<xml_diff>
--- a/data/2025/03-arges/13169-pitesti/budget_file.xlsx
+++ b/data/2025/03-arges/13169-pitesti/budget_file.xlsx
@@ -7282,41 +7282,39 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="3" t="inlineStr">
+      <c r="A237" s="5" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B237" s="3" t="inlineStr">
+      <c r="B237" s="5" t="inlineStr">
         <is>
           <t>70.02</t>
         </is>
       </c>
-      <c r="C237" s="3" t="inlineStr">
+      <c r="C237" s="5" t="inlineStr">
         <is>
           <t>Cheltuieli curente</t>
         </is>
       </c>
-      <c r="D237" s="3" t="n"/>
-      <c r="E237" s="3" t="n">
+      <c r="D237" s="5" t="n"/>
+      <c r="E237" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="F237" s="3" t="inlineStr">
+      <c r="F237" s="5" t="inlineStr">
         <is>
           <t>expense_economic</t>
         </is>
       </c>
-      <c r="G237" s="4" t="n">
-        <v>103918</v>
-      </c>
-      <c r="H237" s="3" t="inlineStr">
-        <is>
-          <t>llm:gemini-3.6-flash</t>
-        </is>
-      </c>
-      <c r="I237" s="3" t="inlineStr">
-        <is>
-          <t>duplicate of p8 with different values; cell re-read from image (unverified transcription)</t>
+      <c r="G237" s="7" t="n"/>
+      <c r="H237" s="5" t="inlineStr">
+        <is>
+          <t>ocr</t>
+        </is>
+      </c>
+      <c r="I237" s="5" t="inlineStr">
+        <is>
+          <t>unparseable cell '59.316 59.316' in column total_2026; duplicate of p8 with different values</t>
         </is>
       </c>
     </row>
@@ -7436,31 +7434,31 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" t="inlineStr">
+      <c r="A241" s="5" t="inlineStr">
         <is>
           <t>79.02.81.02</t>
         </is>
       </c>
-      <c r="C241" s="8" t="inlineStr">
+      <c r="B241" s="5" t="n"/>
+      <c r="C241" s="6" t="inlineStr">
         <is>
           <t>Partea a V-a ACTIUNI ECONOMICE COMBUSTIBILI ŞI ENERGIE</t>
         </is>
       </c>
-      <c r="E241" t="n">
+      <c r="D241" s="5" t="n"/>
+      <c r="E241" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="F241" t="inlineStr"/>
-      <c r="G241" s="2" t="n">
-        <v>24315</v>
-      </c>
-      <c r="H241" t="inlineStr">
-        <is>
-          <t>llm:gemini-3.6-flash</t>
-        </is>
-      </c>
-      <c r="I241" t="inlineStr">
-        <is>
-          <t>cell re-read from image (unverified transcription)</t>
+      <c r="F241" s="5" t="inlineStr"/>
+      <c r="G241" s="7" t="n"/>
+      <c r="H241" s="5" t="inlineStr">
+        <is>
+          <t>ocr</t>
+        </is>
+      </c>
+      <c r="I241" s="5" t="inlineStr">
+        <is>
+          <t>unparseable cell '89.902 24.315' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -7544,60 +7542,60 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" t="inlineStr">
+      <c r="A245" s="5" t="inlineStr">
         <is>
           <t>84.02.01</t>
         </is>
       </c>
-      <c r="C245" s="8" t="inlineStr">
+      <c r="B245" s="5" t="n"/>
+      <c r="C245" s="6" t="inlineStr">
         <is>
           <t>TRANSPORTURI Cheltuieli curente</t>
         </is>
       </c>
-      <c r="E245" t="n">
+      <c r="D245" s="5" t="n"/>
+      <c r="E245" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="F245" t="inlineStr"/>
-      <c r="G245" s="2" t="n">
-        <v>65587</v>
-      </c>
-      <c r="H245" t="inlineStr">
-        <is>
-          <t>llm:gemini-3.6-flash</t>
-        </is>
-      </c>
-      <c r="I245" t="inlineStr">
-        <is>
-          <t>cell re-read from image (unverified transcription)</t>
+      <c r="F245" s="5" t="inlineStr"/>
+      <c r="G245" s="7" t="n"/>
+      <c r="H245" s="5" t="inlineStr">
+        <is>
+          <t>ocr</t>
+        </is>
+      </c>
+      <c r="I245" s="5" t="inlineStr">
+        <is>
+          <t>unparseable cell '65.587 65.587' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="246">
-      <c r="A246" t="inlineStr">
+      <c r="A246" s="5" t="inlineStr">
         <is>
           <t>10.20</t>
         </is>
       </c>
-      <c r="C246" s="8" t="inlineStr">
+      <c r="B246" s="5" t="n"/>
+      <c r="C246" s="6" t="inlineStr">
         <is>
           <t>Titlul I Cheltuieli de personal</t>
         </is>
       </c>
-      <c r="E246" t="n">
+      <c r="D246" s="5" t="n"/>
+      <c r="E246" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="F246" t="inlineStr"/>
-      <c r="G246" s="2" t="n">
-        <v>27249</v>
-      </c>
-      <c r="H246" t="inlineStr">
-        <is>
-          <t>llm:gemini-3.6-flash</t>
-        </is>
-      </c>
-      <c r="I246" t="inlineStr">
-        <is>
-          <t>cell re-read from image (unverified transcription)</t>
+      <c r="F246" s="5" t="inlineStr"/>
+      <c r="G246" s="7" t="n"/>
+      <c r="H246" s="5" t="inlineStr">
+        <is>
+          <t>ocr</t>
+        </is>
+      </c>
+      <c r="I246" s="5" t="inlineStr">
+        <is>
+          <t>unparseable cell '12.852 13.580' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -7633,37 +7631,35 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="3" t="inlineStr">
+      <c r="A248" s="5" t="inlineStr">
         <is>
           <t>59</t>
         </is>
       </c>
-      <c r="B248" s="3" t="inlineStr">
+      <c r="B248" s="5" t="inlineStr">
         <is>
           <t>70.02</t>
         </is>
       </c>
-      <c r="C248" s="3" t="inlineStr"/>
-      <c r="D248" s="3" t="n"/>
-      <c r="E248" s="3" t="n">
+      <c r="C248" s="5" t="inlineStr"/>
+      <c r="D248" s="5" t="n"/>
+      <c r="E248" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="F248" s="3" t="inlineStr">
+      <c r="F248" s="5" t="inlineStr">
         <is>
           <t>expense_economic</t>
         </is>
       </c>
-      <c r="G248" s="4" t="n">
-        <v>18890</v>
-      </c>
-      <c r="H248" s="3" t="inlineStr">
-        <is>
-          <t>llm:gemini-3.6-flash</t>
-        </is>
-      </c>
-      <c r="I248" s="3" t="inlineStr">
-        <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL XI ALTE CHELTUIELI'; cell re-read from image (unverified transcription)</t>
+      <c r="G248" s="7" t="n"/>
+      <c r="H248" s="5" t="inlineStr">
+        <is>
+          <t>ocr</t>
+        </is>
+      </c>
+      <c r="I248" s="5" t="inlineStr">
+        <is>
+          <t>unparseable cell '39.000 155' in column total_2026; name mismatch vs nomenclator (0%): '' vs 'TITLUL XI ALTE CHELTUIELI'</t>
         </is>
       </c>
     </row>
@@ -7845,17 +7841,15 @@
           <t>expense_functional</t>
         </is>
       </c>
-      <c r="G255" s="7" t="n">
-        <v>155037</v>
-      </c>
+      <c r="G255" s="7" t="n"/>
       <c r="H255" s="5" t="inlineStr">
         <is>
-          <t>llm:gemini-3.6-flash</t>
+          <t>ocr</t>
         </is>
       </c>
       <c r="I255" s="5" t="inlineStr">
         <is>
-          <t>code 61.70 (expense_functional) not in nomenclator; cell re-read from image (unverified transcription)</t>
+          <t>unparseable cell '155.037 148.994' in column total_2026; code 61.70 (expense_functional) not in nomenclator</t>
         </is>
       </c>
     </row>
@@ -7945,31 +7939,31 @@
       </c>
     </row>
     <row r="259">
-      <c r="A259" t="inlineStr">
+      <c r="A259" s="5" t="inlineStr">
         <is>
           <t>50.02.51.02</t>
         </is>
       </c>
-      <c r="C259" s="8" t="inlineStr">
+      <c r="B259" s="5" t="n"/>
+      <c r="C259" s="6" t="inlineStr">
         <is>
           <t>Partea I SERVICII PUBLICE GENERALE AUTORITÅTI PUBLICE ŞI ACTIUNI EXTERNE Titlul X Proiecte cu finanțare din fonduri externe nerambursabile aferente cadrului financiar 2014-2020</t>
         </is>
       </c>
-      <c r="E259" t="n">
+      <c r="D259" s="5" t="n"/>
+      <c r="E259" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="F259" t="inlineStr"/>
-      <c r="G259" s="2" t="n">
-        <v>2757</v>
-      </c>
-      <c r="H259" t="inlineStr">
-        <is>
-          <t>llm:gemini-3.6-flash</t>
-        </is>
-      </c>
-      <c r="I259" t="inlineStr">
-        <is>
-          <t>cell re-read from image (unverified transcription)</t>
+      <c r="F259" s="5" t="inlineStr"/>
+      <c r="G259" s="7" t="n"/>
+      <c r="H259" s="5" t="inlineStr">
+        <is>
+          <t>ocr</t>
+        </is>
+      </c>
+      <c r="I259" s="5" t="inlineStr">
+        <is>
+          <t>unparseable cell '2.785 2.757' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -35182,7 +35176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -35228,7 +35222,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -35241,38 +35235,28 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>11.02</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>48.02</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>LLM re-read 5 rows for 11.02 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>name mismatch vs nomenclator (18%): 'VENITURI PROPRII' vs 'Sume primite de la UE/alti donatori in c'</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>V6_repair</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>33.02</t>
-        </is>
+        <v>3</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -35281,27 +35265,27 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>LLM re-read 6 rows for 33.02 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>unparseable cell '61.022 50.896' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>V6_repair</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>35.02</t>
+          <t>11.02</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -35311,27 +35295,27 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>LLM re-read 2 rows for 35.02 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>11.02 total_2026: parent 135.177,00 != sum(children) 13.000,00 (4 children)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>V6_repair</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>42.02</t>
+          <t>33.02</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -35341,27 +35325,27 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>LLM re-read 19 rows for 42.02 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>33.02 total_2026: parent 1.658,00 != sum(children) 1.653,00 (5 children)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>V6_repair</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>42.02.89</t>
+          <t>35.02</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -35371,28 +35355,23 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>LLM re-read 3 rows for 42.02.89 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>35.02 total_2026: parent 6.281,00 != sum(children) 6.259,00 (1 children)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>V6_repair</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>45.02.48</t>
-        </is>
+        <v>4</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -35401,107 +35380,137 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>LLM re-read 2 rows for 45.02.48 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>unparseable cell '6.259 0' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>4</v>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>35.02.03</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>unparseable-cell pass p4: 0 cells recovered</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Incasari din valorificarea bunurilor con'</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>36.02.01</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>unparseable-cell pass p5: 0 cells recovered</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Venituri din aplicarea prescriptiei exti'</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>V6_repair</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>info</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>7</v>
+        <v>4</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>total_2026</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>unparseable-cell pass p7: 0 cells recovered</t>
+          <t>unparseable cell 'x 136.281' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>V6_repair</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>info</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>42.02</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>total_2026</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>unparseable-cell pass p8: 7 cells recovered</t>
+          <t>42.02 total_2026: parent 323.401,00 != sum(children) 19.422,00 (18 children)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9</v>
+        <v>5</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>42.02.21</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>unparseable-cell pass p9: 0 cells recovered</t>
+          <t>name mismatch vs nomenclator (42%): 'Finantarea drepturilor acordate persoane' vs 'Alte drepturi pentru dizabilitate și ado'</t>
         </is>
       </c>
     </row>
@@ -35517,16 +35526,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>48.02</t>
+          <t>42.02.80</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (18%): 'VENITURI PROPRII' vs 'Sume primite de la UE/alti donatori in c'</t>
+          <t>name mismatch vs nomenclator (38%): 'fonduri externe nerambursabile (FEN) pos' vs 'Subvenții de la bugetul de stat pentru d'</t>
         </is>
       </c>
     </row>
@@ -35542,7 +35551,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -35551,7 +35560,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>unparseable cell '61.022 50.896' in column total_2026</t>
+          <t>unparseable cell '149.707 134.230' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -35567,11 +35576,11 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>11.02</t>
+          <t>42.02.89</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -35581,14 +35590,14 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>11.02 total_2026: parent 135.177,00 != sum(children) 13.000,00 (4 children)</t>
+          <t>42.02.89 total_2026: parent 125.514,00 != sum(children) 105.474,00 (2 children)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>V4_hierarchy</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -35597,12 +35606,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>33.02</t>
-        </is>
+        <v>5</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -35611,7 +35615,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>33.02 total_2026: parent 1.658,00 != sum(children) 1.653,00 (5 children)</t>
+          <t>unparseable cell '20.040 2.973' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -35627,11 +35631,11 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>35.02</t>
+          <t>45.02.48</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -35641,32 +35645,32 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>35.02 total_2026: parent 6.281,00 != sum(children) 6.259,00 (1 children)</t>
+          <t>45.02.48 total_2026: parent 19.436,00 != sum(children) 17.698,00 (1 children)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+        <v>6</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>48.02.01</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>unparseable cell '6.259 0' in column total_2026</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Fondul European de Dezvoltare Regională '</t>
         </is>
       </c>
     </row>
@@ -35682,16 +35686,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>35.02.03</t>
+          <t>48.02.01.01</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Incasari din valorificarea bunurilor con'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Sume primite in contul platilor efectuat'</t>
         </is>
       </c>
     </row>
@@ -35707,71 +35711,66 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>36.02.01</t>
+          <t>48.02.01.02</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Venituri din aplicarea prescriptiei exti'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Sume primite in contul platilor efectuat'</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+        <v>6</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>48.02.01.03</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>unparseable cell 'x 136.281' in column total_2026</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Prefinantare'</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>V4_hierarchy</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>42.02</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>48.02.02</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>42.02 total_2026: parent 323.401,00 != sum(children) 19.422,00 (18 children)</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Fondul Social European (FSE)'</t>
         </is>
       </c>
     </row>
@@ -35787,16 +35786,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>42.02.21</t>
+          <t>48.02.02.01</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (42%): 'Finantarea drepturilor acordate persoane' vs 'Alte drepturi pentru dizabilitate și ado'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Sume primite in contul platilor efectuat'</t>
         </is>
       </c>
     </row>
@@ -35812,133 +35811,123 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>42.02.80</t>
+          <t>48.02.02.02</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (38%): 'fonduri externe nerambursabile (FEN) pos' vs 'Subvenții de la bugetul de stat pentru d'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Sume primite in contul platilor efectuat'</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>5</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+        <v>6</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>48.02.02.03</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>unparseable cell '149.707 134.230' in column total_2026</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Prefinantare'</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>V4_hierarchy</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>42.02.89</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>48.02.32</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>42.02.89 total_2026: parent 125.514,00 != sum(children) 105.474,00 (2 children)</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Fondul pentru relații bilaterale aferent'</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+        <v>6</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>48.02.32.01</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>unparseable cell '20.040 2.973' in column total_2026</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Sume primite în contul plăţilor efectuat'</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>V4_hierarchy</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>45.02.48</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>48.02.32.02</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>45.02.48 total_2026: parent 19.436,00 != sum(children) 17.698,00 (1 children)</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Sume primite in contul platilor efectuat'</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -35947,23 +35936,23 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>48.02.01</t>
+          <t>49.02</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Fondul European de Dezvoltare Regională '</t>
+          <t>duplicate of p7 with different values</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -35972,16 +35961,16 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>48.02.01.01</t>
+          <t>01</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Sume primite in contul platilor efectuat'</t>
+          <t>duplicate of p7 with different values</t>
         </is>
       </c>
     </row>
@@ -35997,23 +35986,23 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>48.02.01.02</t>
+          <t>54.02</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Sume primite in contul platilor efectuat'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Alte servicii publice generale'</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -36022,23 +36011,23 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>48.02.01.03</t>
+          <t>01</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Prefinantare'</t>
+          <t>duplicate of p7 with different values</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -36047,23 +36036,23 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>48.02.02</t>
+          <t>01</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Fondul Social European (FSE)'</t>
+          <t>duplicate of p7 with different values</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -36072,48 +36061,48 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>48.02.02.01</t>
+          <t>01</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Sume primite in contul platilor efectuat'</t>
+          <t>duplicate of p7 with different values</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V1_code</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>48.02.02.02</t>
+          <t>10.20</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Sume primite in contul platilor efectuat'</t>
+          <t>code 10.20 (expense_functional) not in nomenclator</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -36122,23 +36111,23 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>48.02.02.03</t>
+          <t>01</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Prefinantare'</t>
+          <t>duplicate of p7 with different values</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -36147,23 +36136,23 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>48.02.32</t>
+          <t>01</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Fondul pentru relații bilaterale aferent'</t>
+          <t>duplicate of p7 with different values</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -36172,53 +36161,53 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>48.02.32.01</t>
+          <t>01</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Sume primite în contul plăţilor efectuat'</t>
+          <t>duplicate of p7 with different values</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>6</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>48.02.32.02</t>
+        <v>7</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Sume primite in contul platilor efectuat'</t>
+          <t>unparseable cell '50.320 23.000' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V1_code</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -36226,12 +36215,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>49.02</t>
+          <t>20.51</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>duplicate of p7 with different values</t>
+          <t>code 20.51 (expense_functional) not in nomenclator</t>
         </is>
       </c>
     </row>
@@ -36247,7 +36236,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -36263,25 +36252,25 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V1_code</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>54.02</t>
+          <t>10.20</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Alte servicii publice generale'</t>
+          <t>code 10.20 (expense_functional) not in nomenclator</t>
         </is>
       </c>
     </row>
@@ -36297,11 +36286,11 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>10.20</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -36313,7 +36302,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -36322,16 +36311,16 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>57</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>duplicate of p7 with different values</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL IX  ASISTENTA SOCIALA'</t>
         </is>
       </c>
     </row>
@@ -36347,11 +36336,11 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>59</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -36363,32 +36352,32 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>V1_code</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>10.20</t>
+          <t>01</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>code 10.20 (expense_functional) not in nomenclator</t>
+          <t>duplicate of p7 with different values</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -36397,41 +36386,41 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>59</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>duplicate of p7 with different values</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL XI ALTE CHELTUIELI'</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V1_code</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>74.02.01</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>duplicate of p7 with different values</t>
+          <t>code 74.02.01 (expense_functional) not in nomenclator</t>
         </is>
       </c>
     </row>
@@ -36441,22 +36430,22 @@
           <t>V7_hygiene</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>warning</t>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>7</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>01</t>
+        <v>8</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>duplicate of p7 with different values</t>
+          <t>unparseable cell '59.316 59.316' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -36466,47 +36455,47 @@
           <t>V7_hygiene</t>
         </is>
       </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>7</v>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+        <v>8</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>unparseable cell '50.320 23.000' in column total_2026</t>
+          <t>duplicate of p8 with different values</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>V1_code</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>20.51</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>code 20.51 (expense_functional) not in nomenclator</t>
+          <t>duplicate of p8 with different values</t>
         </is>
       </c>
     </row>
@@ -36526,24 +36515,24 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>55</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>duplicate of p7 with different values</t>
+          <t>duplicate of p8 with different values</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>V1_code</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -36551,12 +36540,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>10.20</t>
+          <t>59</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>code 10.20 (expense_functional) not in nomenclator</t>
+          <t>duplicate of p8 with different values</t>
         </is>
       </c>
     </row>
@@ -36566,47 +36555,47 @@
           <t>V7_hygiene</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>warning</t>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C54" t="n">
         <v>8</v>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>10.20</t>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>duplicate of p7 with different values</t>
+          <t>unparseable cell '89.902 24.315' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C55" t="n">
         <v>8</v>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>57</t>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL IX  ASISTENTA SOCIALA'</t>
+          <t>unparseable cell '65.587 65.587' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -36616,22 +36605,22 @@
           <t>V7_hygiene</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>warning</t>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C56" t="n">
         <v>8</v>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>59</t>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>duplicate of p7 with different values</t>
+          <t>unparseable cell '12.852 13.580' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -36641,22 +36630,22 @@
           <t>V7_hygiene</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>warning</t>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C57" t="n">
         <v>8</v>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>01</t>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>duplicate of p7 with different values</t>
+          <t>unparseable cell '39.000 155' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -36688,7 +36677,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>V1_code</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -36699,26 +36688,26 @@
       <c r="C59" t="n">
         <v>8</v>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>74.02.01</t>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>code 74.02.01 (expense_functional) not in nomenclator</t>
+          <t>unparseable cell '155.037 148.994' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V1_code</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -36726,24 +36715,24 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>61.70</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>duplicate of p8 with different values</t>
+          <t>code 61.70 (expense_functional) not in nomenclator</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -36751,17 +36740,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>72</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL XVII ACTIVE FINANCIARE'</t>
         </is>
       </c>
     </row>
@@ -36771,123 +36755,123 @@
           <t>V7_hygiene</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>warning</t>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C62" t="n">
         <v>8</v>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>20</t>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>duplicate of p8 with different values</t>
+          <t>unparseable cell '2.785 2.757' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>61.02</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>duplicate of p8 with different values</t>
+          <t>61.02 total_2026: parent 4.694,00 != sum(children) 3.925,00 (1 children)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>65.02</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>duplicate of p8 with different values</t>
+          <t>65.02 total_2026: parent 194.414,00 != sum(children) 16.657,00 (1 children)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>79.02.81.02</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>58</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>duplicate of p9 with different values</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>V6_repair</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>info</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>8</v>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>84.02.01</t>
-        </is>
+        <v>9</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -36896,44 +36880,39 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>unparseable cell '36.752 36.752' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>10.20</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>70</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>duplicate of p9 with different values</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -36942,36 +36921,36 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>71</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL XI ALTE CHELTUIELI'</t>
+          <t>duplicate of p9 with different values</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>V6_repair</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>info</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>74.02</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -36981,62 +36960,57 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>74.02 total_2026: parent 50.840,00 != sum(children) 20.257,00 (1 children)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>V1_code</t>
-        </is>
-      </c>
-      <c r="B70" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>61.70</t>
+          <t>71</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>code 61.70 (expense_functional) not in nomenclator</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>61.70</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>56</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>name mismatch vs nomenclator (45%): '56 Programe finantate din Fondul Europea' vs 'Titlul VIII PROIECTE CU FINANTARE DIN FO'</t>
         </is>
       </c>
     </row>
@@ -37052,113 +37026,98 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>56</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL XVII ACTIVE FINANCIARE'</t>
+          <t>name mismatch vs nomenclator (45%): '56 Programe finantate din Fondul Europea' vs 'Titlul VIII PROIECTE CU FINANTARE DIN FO'</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>50.02.51.02</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>56</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>name mismatch vs nomenclator (45%): '56 Programe finantate din Fondul Europea' vs 'Titlul VIII PROIECTE CU FINANTARE DIN FO'</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>V4_hierarchy</t>
-        </is>
-      </c>
-      <c r="B74" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>61.02</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>71</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>61.02 total_2026: parent 4.694,00 != sum(children) 3.925,00 (1 children)</t>
+          <t>duplicate of p14 with different values</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>V4_hierarchy</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
           <t>65.02</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>total_2026</t>
-        </is>
-      </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>65.02 total_2026: parent 194.414,00 != sum(children) 16.657,00 (1 children)</t>
+          <t>name mismatch vs nomenclator (26%): 'Cap. 65.02 „Învățământ”, din care:' vs 'Cheltuieli aferente programelor cu finan'</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -37167,48 +37126,48 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>84.02</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>duplicate of p9 with different values</t>
+          <t>name mismatch vs nomenclator (50%): 'Cap. 84.02 „Transporturi”, din care:' vs 'Transporturi'</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B77" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>9</v>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+        <v>22</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>unparseable cell '36.752 36.752' in column total_2026</t>
+          <t>name mismatch vs nomenclator (34%): 'Venituri proprii' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -37217,23 +37176,23 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>duplicate of p9 with different values</t>
+          <t>name mismatch vs nomenclator (34%): 'Venituri proprii' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -37242,46 +37201,41 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>51.02</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>duplicate of p9 with different values</t>
+          <t>name mismatch vs nomenclator (38%): 'CAPITOLUL 51.02 Autorități executive' vs 'Transferuri de capital'</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>V4_hierarchy</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>74.02</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>74.02 total_2026: parent 50.840,00 != sum(children) 20.257,00 (1 children)</t>
+          <t>name mismatch vs nomenclator (35%): 'Renovare energetică Şcoala Gimnazială Ni' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37297,16 +37251,16 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37322,16 +37276,16 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (45%): '56 Programe finantate din Fondul Europea' vs 'Titlul VIII PROIECTE CU FINANTARE DIN FO'</t>
+          <t>name mismatch vs nomenclator (38%): 'Renovare energetică Liceul de Arte Dinu ' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37347,16 +37301,16 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (45%): '56 Programe finantate din Fondul Europea' vs 'Titlul VIII PROIECTE CU FINANTARE DIN FO'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37372,23 +37326,23 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (45%): '56 Programe finantate din Fondul Europea' vs 'Titlul VIII PROIECTE CU FINANTARE DIN FO'</t>
+          <t>name mismatch vs nomenclator (32%): 'Renovare energetică Grădinița cu Program' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -37397,16 +37351,16 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>duplicate of p14 with different values</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37422,16 +37376,16 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>65.02</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (26%): 'Cap. 65.02 „Învățământ”, din care:' vs 'Cheltuieli aferente programelor cu finan'</t>
+          <t>name mismatch vs nomenclator (33%): 'Eficientizare energetică Şcoala Gimnazia' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37447,16 +37401,16 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>84.02</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (50%): 'Cap. 84.02 „Transporturi”, din care:' vs 'Transporturi'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37472,7 +37426,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -37481,7 +37435,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (34%): 'Venituri proprii' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (41%): 'Eficientizare energetică Școala Gimnazia' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37497,7 +37451,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -37506,7 +37460,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (34%): 'Venituri proprii' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (38%): 'Eficientizare energetică Grădinița cu Pr' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37522,16 +37476,16 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>51.02</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (38%): 'CAPITOLUL 51.02 Autorități executive' vs 'Transferuri de capital'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37556,7 +37510,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (35%): 'Renovare energetică Şcoala Gimnazială Ni' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (40%): 'Eficientizare energetică Şcoala Gimnazia' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37581,7 +37535,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (36%): 'Eficientizare energetică Şcoala Gimnazia' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37606,7 +37560,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (38%): 'Renovare energetică Liceul de Arte Dinu ' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
@@ -37626,12 +37580,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>55</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (26%): 'Sală de educație fizică școlară - Proiec' vs 'TITLUL VII ALTE TRANSFERURI'</t>
         </is>
       </c>
     </row>
@@ -37651,12 +37605,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (32%): 'Renovare energetică Grădinița cu Program' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (40%): 'Nicolae Bălcescu" Documentație în vedere' vs 'Titlul XII „Proiecte cu finanțare din su'</t>
         </is>
       </c>
     </row>
@@ -37676,12 +37630,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (12%): 'Călinescu"' vs 'Titlul XII „Proiecte cu finanțare din su'</t>
         </is>
       </c>
     </row>
@@ -37701,12 +37655,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>55</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (33%): 'Eficientizare energetică Şcoala Gimnazia' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (25%): 'municipiul Pitești, B-dul Petrochimiștil' vs 'TITLUL VII ALTE TRANSFERURI'</t>
         </is>
       </c>
     </row>
@@ -37726,12 +37680,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (25%): 'Înlocuire gard și sistematizare interioa' vs 'TITLUL IV SUBVENTII'</t>
         </is>
       </c>
     </row>
@@ -37751,12 +37705,12 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (41%): 'Eficientizare energetică Școala Gimnazia' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (43%): 'Viitorul"' vs 'TITLUL IV SUBVENTII'</t>
         </is>
       </c>
     </row>
@@ -37776,12 +37730,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (38%): 'Eficientizare energetică Grădinița cu Pr' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (35%): 'Teren de sport cu suprafață modulară Şco' vs 'TITLUL V FONDURI DE REZERVA'</t>
         </is>
       </c>
     </row>
@@ -37801,12 +37755,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL V FONDURI DE REZERVA'</t>
         </is>
       </c>
     </row>
@@ -37826,12 +37780,12 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (40%): 'Eficientizare energetică Şcoala Gimnazia' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (30%): 'Teren de sport cu suprafață modulară Şco' vs 'TITLUL V FONDURI DE REZERVA'</t>
         </is>
       </c>
     </row>
@@ -37851,12 +37805,12 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (36%): 'Eficientizare energetică Şcoala Gimnazia' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (31%): 'Teren de sport cu suprafață modulară Şco' vs 'TITLUL V FONDURI DE REZERVA'</t>
         </is>
       </c>
     </row>
@@ -37876,12 +37830,12 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL V FONDURI DE REZERVA'</t>
         </is>
       </c>
     </row>
@@ -37901,12 +37855,12 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (26%): 'Sală de educație fizică școlară - Proiec' vs 'TITLUL VII ALTE TRANSFERURI'</t>
+          <t>name mismatch vs nomenclator (29%): 'Teren de sport cu suprafață modulară Şco' vs 'TITLUL V FONDURI DE REZERVA'</t>
         </is>
       </c>
     </row>
@@ -37922,23 +37876,23 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>81.02</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (40%): 'Nicolae Bălcescu" Documentație în vedere' vs 'Titlul XII „Proiecte cu finanțare din su'</t>
+          <t>name mismatch vs nomenclator (40%): 'Cap. 81.02 „Combustibili și energie”' vs 'Rambursari de credite interne'</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -37947,23 +37901,23 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>71</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (12%): 'Călinescu"' vs 'Titlul XII „Proiecte cu finanțare din su'</t>
+          <t>duplicate of p30 with different values</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -37972,23 +37926,23 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>71</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (25%): 'municipiul Pitești, B-dul Petrochimiștil' vs 'TITLUL VII ALTE TRANSFERURI'</t>
+          <t>duplicate of p30 with different values</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -37997,289 +37951,14 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>71</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
-        <is>
-          <t>name mismatch vs nomenclator (25%): 'Înlocuire gard și sistematizare interioa' vs 'TITLUL IV SUBVENTII'</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="C110" t="n">
-        <v>25</v>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>name mismatch vs nomenclator (43%): 'Viitorul"' vs 'TITLUL IV SUBVENTII'</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="C111" t="n">
-        <v>25</v>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>name mismatch vs nomenclator (35%): 'Teren de sport cu suprafață modulară Şco' vs 'TITLUL V FONDURI DE REZERVA'</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="C112" t="n">
-        <v>25</v>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL V FONDURI DE REZERVA'</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="C113" t="n">
-        <v>25</v>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>name mismatch vs nomenclator (30%): 'Teren de sport cu suprafață modulară Şco' vs 'TITLUL V FONDURI DE REZERVA'</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="C114" t="n">
-        <v>25</v>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>name mismatch vs nomenclator (31%): 'Teren de sport cu suprafață modulară Şco' vs 'TITLUL V FONDURI DE REZERVA'</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="C115" t="n">
-        <v>25</v>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'TITLUL V FONDURI DE REZERVA'</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="C116" t="n">
-        <v>25</v>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>name mismatch vs nomenclator (29%): 'Teren de sport cu suprafață modulară Şco' vs 'TITLUL V FONDURI DE REZERVA'</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="C117" t="n">
-        <v>29</v>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>81.02</t>
-        </is>
-      </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>name mismatch vs nomenclator (40%): 'Cap. 81.02 „Combustibili și energie”' vs 'Rambursari de credite interne'</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="C118" t="n">
-        <v>31</v>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>71</t>
-        </is>
-      </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>duplicate of p30 with different values</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="C119" t="n">
-        <v>31</v>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>71</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>duplicate of p30 with different values</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="C120" t="n">
-        <v>32</v>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>71</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
         <is>
           <t>duplicate of p31 with different values</t>
         </is>
@@ -38296,7 +37975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -38318,7 +37997,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Documente</t>
+          <t>Schema calitate</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -38328,72 +38007,242 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>Linii de date</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>403</v>
+          <t>Metrica de calitate</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>observed_strict_line_rate</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Linii fara probleme</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>308</v>
+          <t>Recall masurat</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>nu</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>% curat</t>
+          <t>Documente</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>76.40000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Erori</t>
+          <t>Linii de date</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>21</v>
+        <v>403</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Avertismente</t>
+          <t>Linii strict verificate</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>86</v>
+        <v>308</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Modele LLM folosite</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>gemini-3.6-flash</t>
-        </is>
+          <t>% linii strict verificate</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>76.40000000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
+          <t>Celule numerice</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Celule numerice strict verificate</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>% celule numerice strict verificate</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>83.8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Pagini asteptate</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Pagini selectate</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Pagini procesate</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>PDF complet</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Linii fara probleme</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>% curat</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>76.40000000000001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Erori</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Avertismente</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Informatii</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Schema publicare</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Bundle conversie</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>7de1ee8a21fc7bf4aababc1e</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>SHA-256 PDF sursa</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>040ccefe38f4b3bc096be69bbdb87a73afae9c2a08bbc4f7c3edd8401a2e6715</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Modele LLM folosite</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>gemini-3.6-flash</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
           <t>— Anexa (de la pagina 3)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>local, pag. 3-38, 1554 linii</t>
         </is>

</xml_diff>